<commit_message>
mise à jour de liens
Ajout des liens pour CRM
</commit_message>
<xml_diff>
--- a/Images/Tableau de synthèse - Debaisieux Matthieu.xlsx
+++ b/Images/Tableau de synthèse - Debaisieux Matthieu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dbf579e00f6a4d0d/Desktop/Codage/Dossier pro/Images/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{48AB5734-CBC2-4D0C-8D3C-F0EC87EAF822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{841F3384-67E0-4145-9660-0F08ED2725F1}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{48AB5734-CBC2-4D0C-8D3C-F0EC87EAF822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{210C5662-09F9-4DFD-A8FF-99DAE6AD875A}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -168,9 +168,6 @@
     <t>15/06/26 au 19/06/26</t>
   </si>
   <si>
-    <t xml:space="preserve">Élaboration du dossier de cadrage, de planification et de découpage des tâches, pour un projet de CRM </t>
-  </si>
-  <si>
     <t>Réalisations en milieu professionnel en cours de première année</t>
   </si>
   <si>
@@ -205,6 +202,12 @@
   </si>
   <si>
     <t>Création d'un site web capable d’analyser une URL fournie par un utilisateur afin de générer un rapport SEO simplifié, clair et pédagogique.</t>
+  </si>
+  <si>
+    <t>15/06/26 au 19/06/26 et 7/09/26 au 11/09/26</t>
+  </si>
+  <si>
+    <t>Élaboration d'un outil de gestion pour un club de volley : première semaine dans un pôle gestion de projet, la seconde dans un pôle modélisation de base de donnée(merise)/RGPD et backend</t>
   </si>
 </sst>
 </file>
@@ -920,6 +923,48 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -958,48 +1003,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1017,10 +1020,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1331,29 +1330,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
-      <c r="F1" s="75"/>
-      <c r="G1" s="75"/>
-      <c r="H1" s="75"/>
-      <c r="I1" s="75"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
-      <c r="R1" s="75"/>
-      <c r="S1" s="75"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
       <c r="T1" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="U1" s="17"/>
       <c r="V1" s="18"/>
@@ -1389,142 +1388,142 @@
       <c r="X2" s="22"/>
     </row>
     <row r="3" spans="1:59" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="80" t="s">
-        <v>44</v>
-      </c>
-      <c r="B3" s="86"/>
-      <c r="C3" s="86"/>
-      <c r="D3" s="86"/>
-      <c r="E3" s="86"/>
-      <c r="F3" s="86"/>
-      <c r="G3" s="86"/>
-      <c r="H3" s="86"/>
-      <c r="I3" s="86"/>
-      <c r="J3" s="86"/>
-      <c r="K3" s="86"/>
-      <c r="L3" s="86"/>
-      <c r="M3" s="86"/>
-      <c r="N3" s="86"/>
-      <c r="O3" s="86"/>
-      <c r="P3" s="86"/>
-      <c r="Q3" s="87"/>
-      <c r="R3" s="76" t="s">
+      <c r="A3" s="67" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="73"/>
+      <c r="C3" s="73"/>
+      <c r="D3" s="73"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="73"/>
+      <c r="G3" s="73"/>
+      <c r="H3" s="73"/>
+      <c r="I3" s="73"/>
+      <c r="J3" s="73"/>
+      <c r="K3" s="73"/>
+      <c r="L3" s="73"/>
+      <c r="M3" s="73"/>
+      <c r="N3" s="73"/>
+      <c r="O3" s="73"/>
+      <c r="P3" s="73"/>
+      <c r="Q3" s="74"/>
+      <c r="R3" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="S3" s="77"/>
-      <c r="T3" s="78"/>
-      <c r="U3" s="78"/>
-      <c r="V3" s="78"/>
-      <c r="W3" s="78"/>
-      <c r="X3" s="79"/>
+      <c r="S3" s="64"/>
+      <c r="T3" s="65"/>
+      <c r="U3" s="65"/>
+      <c r="V3" s="65"/>
+      <c r="W3" s="65"/>
+      <c r="X3" s="66"/>
     </row>
     <row r="4" spans="1:59" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="83" t="s">
+      <c r="A4" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="84"/>
-      <c r="C4" s="84"/>
-      <c r="D4" s="84"/>
-      <c r="E4" s="84"/>
-      <c r="F4" s="84"/>
-      <c r="G4" s="84"/>
-      <c r="H4" s="84"/>
-      <c r="I4" s="84"/>
-      <c r="J4" s="84"/>
-      <c r="K4" s="84"/>
-      <c r="L4" s="84"/>
-      <c r="M4" s="84"/>
-      <c r="N4" s="84"/>
-      <c r="O4" s="84"/>
-      <c r="P4" s="84"/>
-      <c r="Q4" s="85"/>
+      <c r="B4" s="71"/>
+      <c r="C4" s="71"/>
+      <c r="D4" s="71"/>
+      <c r="E4" s="71"/>
+      <c r="F4" s="71"/>
+      <c r="G4" s="71"/>
+      <c r="H4" s="71"/>
+      <c r="I4" s="71"/>
+      <c r="J4" s="71"/>
+      <c r="K4" s="71"/>
+      <c r="L4" s="71"/>
+      <c r="M4" s="71"/>
+      <c r="N4" s="71"/>
+      <c r="O4" s="71"/>
+      <c r="P4" s="71"/>
+      <c r="Q4" s="72"/>
       <c r="R4" s="26"/>
       <c r="S4" s="23" t="s">
         <v>4</v>
       </c>
       <c r="T4" s="24"/>
-      <c r="U4" s="67" t="s">
+      <c r="U4" s="81" t="s">
+        <v>44</v>
+      </c>
+      <c r="V4" s="82"/>
+      <c r="W4" s="25" t="s">
         <v>45</v>
-      </c>
-      <c r="V4" s="68"/>
-      <c r="W4" s="25" t="s">
-        <v>46</v>
       </c>
       <c r="X4" s="19"/>
     </row>
     <row r="5" spans="1:59" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="80" t="s">
+      <c r="A5" s="67" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="81"/>
-      <c r="C5" s="81"/>
-      <c r="D5" s="81"/>
-      <c r="E5" s="81"/>
-      <c r="F5" s="81"/>
-      <c r="G5" s="81"/>
-      <c r="H5" s="81"/>
-      <c r="I5" s="81"/>
-      <c r="J5" s="81"/>
-      <c r="K5" s="81"/>
-      <c r="L5" s="81"/>
-      <c r="M5" s="81"/>
-      <c r="N5" s="81"/>
-      <c r="O5" s="81"/>
-      <c r="P5" s="81"/>
-      <c r="Q5" s="81"/>
-      <c r="R5" s="81"/>
-      <c r="S5" s="81"/>
-      <c r="T5" s="81"/>
-      <c r="U5" s="81"/>
-      <c r="V5" s="81"/>
-      <c r="W5" s="81"/>
-      <c r="X5" s="82"/>
+      <c r="B5" s="68"/>
+      <c r="C5" s="68"/>
+      <c r="D5" s="68"/>
+      <c r="E5" s="68"/>
+      <c r="F5" s="68"/>
+      <c r="G5" s="68"/>
+      <c r="H5" s="68"/>
+      <c r="I5" s="68"/>
+      <c r="J5" s="68"/>
+      <c r="K5" s="68"/>
+      <c r="L5" s="68"/>
+      <c r="M5" s="68"/>
+      <c r="N5" s="68"/>
+      <c r="O5" s="68"/>
+      <c r="P5" s="68"/>
+      <c r="Q5" s="68"/>
+      <c r="R5" s="68"/>
+      <c r="S5" s="68"/>
+      <c r="T5" s="68"/>
+      <c r="U5" s="68"/>
+      <c r="V5" s="68"/>
+      <c r="W5" s="68"/>
+      <c r="X5" s="69"/>
     </row>
     <row r="6" spans="1:59" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="72" t="s">
+      <c r="A6" s="86" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="73" t="s">
+      <c r="B6" s="87" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="64" t="s">
+      <c r="C6" s="78" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="65"/>
-      <c r="E6" s="65"/>
-      <c r="F6" s="65"/>
-      <c r="G6" s="65"/>
-      <c r="H6" s="65"/>
-      <c r="I6" s="64" t="s">
+      <c r="D6" s="79"/>
+      <c r="E6" s="79"/>
+      <c r="F6" s="79"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="79"/>
+      <c r="I6" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="J6" s="65"/>
-      <c r="K6" s="65"/>
-      <c r="L6" s="64" t="s">
+      <c r="J6" s="79"/>
+      <c r="K6" s="79"/>
+      <c r="L6" s="78" t="s">
         <v>10</v>
       </c>
-      <c r="M6" s="65"/>
-      <c r="N6" s="65"/>
-      <c r="O6" s="64" t="s">
+      <c r="M6" s="79"/>
+      <c r="N6" s="79"/>
+      <c r="O6" s="78" t="s">
         <v>11</v>
       </c>
-      <c r="P6" s="65"/>
-      <c r="Q6" s="65"/>
-      <c r="R6" s="64" t="s">
+      <c r="P6" s="79"/>
+      <c r="Q6" s="79"/>
+      <c r="R6" s="78" t="s">
         <v>12</v>
       </c>
-      <c r="S6" s="65"/>
-      <c r="T6" s="65"/>
-      <c r="U6" s="66" t="s">
+      <c r="S6" s="79"/>
+      <c r="T6" s="79"/>
+      <c r="U6" s="80" t="s">
         <v>13</v>
       </c>
-      <c r="V6" s="66"/>
-      <c r="W6" s="66"/>
-      <c r="X6" s="66"/>
+      <c r="V6" s="80"/>
+      <c r="W6" s="80"/>
+      <c r="X6" s="80"/>
     </row>
     <row r="7" spans="1:59" s="2" customFormat="1" ht="390.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="72"/>
-      <c r="B7" s="73"/>
+      <c r="A7" s="86"/>
+      <c r="B7" s="87"/>
       <c r="C7" s="47" t="s">
         <v>14</v>
       </c>
@@ -1628,32 +1627,32 @@
       <c r="BG7" s="35"/>
     </row>
     <row r="8" spans="1:59" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="69" t="s">
+      <c r="A8" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="70"/>
-      <c r="C8" s="70"/>
-      <c r="D8" s="70"/>
-      <c r="E8" s="70"/>
-      <c r="F8" s="70"/>
-      <c r="G8" s="70"/>
-      <c r="H8" s="70"/>
-      <c r="I8" s="70"/>
-      <c r="J8" s="70"/>
-      <c r="K8" s="70"/>
-      <c r="L8" s="70"/>
-      <c r="M8" s="70"/>
-      <c r="N8" s="70"/>
-      <c r="O8" s="70"/>
-      <c r="P8" s="70"/>
-      <c r="Q8" s="70"/>
-      <c r="R8" s="70"/>
-      <c r="S8" s="70"/>
-      <c r="T8" s="70"/>
-      <c r="U8" s="70"/>
-      <c r="V8" s="70"/>
-      <c r="W8" s="70"/>
-      <c r="X8" s="71"/>
+      <c r="B8" s="84"/>
+      <c r="C8" s="84"/>
+      <c r="D8" s="84"/>
+      <c r="E8" s="84"/>
+      <c r="F8" s="84"/>
+      <c r="G8" s="84"/>
+      <c r="H8" s="84"/>
+      <c r="I8" s="84"/>
+      <c r="J8" s="84"/>
+      <c r="K8" s="84"/>
+      <c r="L8" s="84"/>
+      <c r="M8" s="84"/>
+      <c r="N8" s="84"/>
+      <c r="O8" s="84"/>
+      <c r="P8" s="84"/>
+      <c r="Q8" s="84"/>
+      <c r="R8" s="84"/>
+      <c r="S8" s="84"/>
+      <c r="T8" s="84"/>
+      <c r="U8" s="84"/>
+      <c r="V8" s="84"/>
+      <c r="W8" s="84"/>
+      <c r="X8" s="85"/>
       <c r="Y8"/>
       <c r="Z8"/>
       <c r="AA8"/>
@@ -1822,21 +1821,19 @@
     </row>
     <row r="11" spans="1:59" s="2" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="B11" s="54" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C11" s="13"/>
-      <c r="D11" s="16"/>
+      <c r="D11" s="37"/>
       <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
+      <c r="F11" s="56"/>
       <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="16"/>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
+      <c r="H11" s="56"/>
+      <c r="I11" s="16"/>
+      <c r="L11" s="40"/>
       <c r="M11" s="16"/>
       <c r="N11" s="16"/>
       <c r="O11" s="41"/>
@@ -1887,10 +1884,10 @@
     </row>
     <row r="12" spans="1:59" s="2" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B12" s="54" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="16"/>
@@ -1952,10 +1949,10 @@
     </row>
     <row r="13" spans="1:59" s="2" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B13" s="54" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="29"/>
@@ -2321,32 +2318,32 @@
       <c r="BG18" s="35"/>
     </row>
     <row r="19" spans="1:59" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A19" s="61" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="62"/>
-      <c r="C19" s="62"/>
-      <c r="D19" s="62"/>
-      <c r="E19" s="62"/>
-      <c r="F19" s="62"/>
-      <c r="G19" s="62"/>
-      <c r="H19" s="62"/>
-      <c r="I19" s="62"/>
-      <c r="J19" s="62"/>
-      <c r="K19" s="62"/>
-      <c r="L19" s="62"/>
-      <c r="M19" s="62"/>
-      <c r="N19" s="62"/>
-      <c r="O19" s="62"/>
-      <c r="P19" s="62"/>
-      <c r="Q19" s="62"/>
-      <c r="R19" s="62"/>
-      <c r="S19" s="62"/>
-      <c r="T19" s="62"/>
-      <c r="U19" s="62"/>
-      <c r="V19" s="62"/>
-      <c r="W19" s="62"/>
-      <c r="X19" s="63"/>
+      <c r="A19" s="75" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" s="76"/>
+      <c r="C19" s="76"/>
+      <c r="D19" s="76"/>
+      <c r="E19" s="76"/>
+      <c r="F19" s="76"/>
+      <c r="G19" s="76"/>
+      <c r="H19" s="76"/>
+      <c r="I19" s="76"/>
+      <c r="J19" s="76"/>
+      <c r="K19" s="76"/>
+      <c r="L19" s="76"/>
+      <c r="M19" s="76"/>
+      <c r="N19" s="76"/>
+      <c r="O19" s="76"/>
+      <c r="P19" s="76"/>
+      <c r="Q19" s="76"/>
+      <c r="R19" s="76"/>
+      <c r="S19" s="76"/>
+      <c r="T19" s="76"/>
+      <c r="U19" s="76"/>
+      <c r="V19" s="76"/>
+      <c r="W19" s="76"/>
+      <c r="X19" s="77"/>
       <c r="Y19"/>
       <c r="Z19"/>
       <c r="AA19"/>
@@ -2385,10 +2382,10 @@
     </row>
     <row r="20" spans="1:59" s="2" customFormat="1" ht="38.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B20" s="54" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="37"/>
@@ -2753,32 +2750,32 @@
       <c r="BG25" s="35"/>
     </row>
     <row r="26" spans="1:59" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A26" s="61" t="s">
-        <v>43</v>
-      </c>
-      <c r="B26" s="62"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="62"/>
-      <c r="E26" s="62"/>
-      <c r="F26" s="62"/>
-      <c r="G26" s="62"/>
-      <c r="H26" s="62"/>
-      <c r="I26" s="62"/>
-      <c r="J26" s="62"/>
-      <c r="K26" s="62"/>
-      <c r="L26" s="62"/>
-      <c r="M26" s="62"/>
-      <c r="N26" s="62"/>
-      <c r="O26" s="62"/>
-      <c r="P26" s="62"/>
-      <c r="Q26" s="62"/>
-      <c r="R26" s="62"/>
-      <c r="S26" s="62"/>
-      <c r="T26" s="62"/>
-      <c r="U26" s="62"/>
-      <c r="V26" s="62"/>
-      <c r="W26" s="62"/>
-      <c r="X26" s="63"/>
+      <c r="A26" s="75" t="s">
+        <v>42</v>
+      </c>
+      <c r="B26" s="76"/>
+      <c r="C26" s="76"/>
+      <c r="D26" s="76"/>
+      <c r="E26" s="76"/>
+      <c r="F26" s="76"/>
+      <c r="G26" s="76"/>
+      <c r="H26" s="76"/>
+      <c r="I26" s="76"/>
+      <c r="J26" s="76"/>
+      <c r="K26" s="76"/>
+      <c r="L26" s="76"/>
+      <c r="M26" s="76"/>
+      <c r="N26" s="76"/>
+      <c r="O26" s="76"/>
+      <c r="P26" s="76"/>
+      <c r="Q26" s="76"/>
+      <c r="R26" s="76"/>
+      <c r="S26" s="76"/>
+      <c r="T26" s="76"/>
+      <c r="U26" s="76"/>
+      <c r="V26" s="76"/>
+      <c r="W26" s="76"/>
+      <c r="X26" s="77"/>
       <c r="Y26"/>
       <c r="Z26"/>
       <c r="AA26"/>
@@ -3107,11 +3104,6 @@
     <row r="76" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A1:S1"/>
-    <mergeCell ref="R3:X3"/>
-    <mergeCell ref="A5:X5"/>
-    <mergeCell ref="A4:Q4"/>
-    <mergeCell ref="A3:Q3"/>
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A19:X19"/>
     <mergeCell ref="R6:T6"/>
@@ -3124,6 +3116,11 @@
     <mergeCell ref="O6:Q6"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="R3:X3"/>
+    <mergeCell ref="A5:X5"/>
+    <mergeCell ref="A4:Q4"/>
+    <mergeCell ref="A3:Q3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -3335,15 +3332,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="191d0fcf-6d89-4c90-807a-10f37b8d7a4c">
@@ -3352,6 +3340,15 @@
     <TaxCatchAll xmlns="9a7dc87b-2be1-4fee-871a-355a79ca984c" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3374,14 +3371,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57628116-2DE7-472D-96A4-5B7B67B2555B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{60914C46-14D0-4134-947D-4237006DD29D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3390,4 +3379,12 @@
     <ds:schemaRef ds:uri="9a7dc87b-2be1-4fee-871a-355a79ca984c"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57628116-2DE7-472D-96A4-5B7B67B2555B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>